<commit_message>
refactor: update ai-audit-log.xlsx and week 5/ai-audit-log.md to match Copy of ai-audit-log.xlsx
</commit_message>
<xml_diff>
--- a/ai-audit-log.xlsx
+++ b/ai-audit-log.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Hanh\FU\RBL\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ASUS\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{12B9848B-E2B0-4C80-8C43-4B05EC6DFC3A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{6CD4E6AE-675A-469C-A36B-A77862246722}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{84C35D15-8A6C-4EDA-8B49-2CCD89DED56E}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{84C35D15-8A6C-4EDA-8B49-2CCD89DED56E}"/>
   </bookViews>
   <sheets>
     <sheet name="Template" sheetId="1" r:id="rId1"/>
@@ -33,6 +33,9 @@
         <xcalcf:feature name="microsoft.com:LET_WF"/>
       </xcalcf:calcFeatures>
     </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
   </extLst>
 </workbook>
 </file>
@@ -40,27 +43,6 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
   <si>
-    <t>Ví dụ: Abstraction</t>
-  </si>
-  <si>
-    <t>“Tôi cần quản lý thông tin sinh viên cho app quản lý điểm. Hãy liệt kê các thuộc tính cần thiết."</t>
-  </si>
-  <si>
-    <t>Ví dụ: Process/Algorithm</t>
-  </si>
-  <si>
-    <t>Ví dụ: Pattern Recognition</t>
-  </si>
-  <si>
-    <t>“So sánh các giải thuật CPU scheduling: FCFS, SJF, Round Robin, Priority. Giải thuật nào tốt nhất?”</t>
-  </si>
-  <si>
-    <t>Ví dụ: Pattern Recognition + Literature Review</t>
-  </si>
-  <si>
-    <t>“Tóm tắt 5 bài báo gần đây nhất về anomaly detection trong IoT sensor data.”</t>
-  </si>
-  <si>
     <t>Giai đoạn/Thành phần DTC</t>
   </si>
   <si>
@@ -73,26 +55,43 @@
     <t>STT</t>
   </si>
   <si>
-    <t>Phản hồi: AI liệt kê 20 thuộc tính.
-Quyết định: Tôi chỉ chọn 10 thuộc tính liên quan đến chức năng đang được yêu cầu từ ứng dụng (CCCD, địa chỉ...) và lược bỏ 10 thuộc tính học thuật vì phù hợp với yêu cầu của ứng dụng</t>
-  </si>
-  <si>
-    <t>"Viết hàm C sắp xếp mảng sinh viên theo điểm số bằng Selection Sort."</t>
-  </si>
-  <si>
-    <t>Phản hồi: AI cung cấp code mẫu.
-Kiểm chứng: Tôi nhận thấy code AI chưa xử lý trường hợp mảng rỗng (Oversimplification). Tôi đã yêu cầu AI tối ưu lại và tự tay bổ sung điều kiện kiểm tra lỗi.</t>
-  </si>
-  <si>
-    <t>Phản hồi: AI response Round Robin là “tốt nhất” vì cân bằng giữa throughput và fairness.
-Kiểm chứng: AI đưa kết luận sai – không có giải thuật “tốt nhất” tuyệt đối (Hallucination). Mỗi giải thuật phù hợp với tình huống/context khác nhau.</t>
-  </si>
-  <si>
-    <t>Phản hồi: AI tóm tắt 5 papers với tên tác giả, năm xuất bản và tóm tắt nội dung.
-Kiểm chứng: Tìm trên Google Scholar: 2/5 papers AI nêu là không tồn tại (fabrication). Tôi đã thay bằng 2 papers mà tôi đã tìm kiếm trên research gates và đã kiểm chứng trên google scholar.</t>
-  </si>
-  <si>
     <t>AI Output</t>
+  </si>
+  <si>
+    <t>"Chúng tôi muốn thay thế đăng nhập Facebook bằng đăng nhập Google trong ứng dụng React + Vite + Node.js (Express). Chúng tôi nên sử dụng nút iframe chính thức của Google hay nút tự thiết kế (custom button) kết hợp với bộ thư viện Google Identity Services Client SDK (initTokenClient)?"</t>
+  </si>
+  <si>
+    <t>AI khuyên nên sử dụng nút Iframe chính thức của Google (google.accounts.id.renderButton) để đảm bảo tính bảo mật cao nhất (sử dụng luồng OIDC ID Token / JWT) và dễ dàng cài đặt tính năng tự động đăng nhập nhanh (Google One Tap).</t>
+  </si>
+  <si>
+    <t>Quyết định cuối cùng và Lý do: Quyết định sử dụng Nút tự thiết kế (Custom Button) + Luồng lấy Access Token (Implicit Flow). Giải pháp này vừa đáp ứng 100% yêu cầu về mặt thẩm mỹ vừa bảo mật tuyệt đối nhờ cơ chế xác thực Access Token trực tiếp từ Server của chúng ta tới máy chủ Google.</t>
+  </si>
+  <si>
+    <t>Abstraction</t>
+  </si>
+  <si>
+    <t>Algorithm</t>
+  </si>
+  <si>
+    <t>"Viết một biểu thức chính quy (regex) và một hàm kiểm tra để xác thực mật khẩu mạnh (tối thiểu 8 ký tự, 1 chữ viết hoa, 1 số, 1 ký tự đặc biệt) và kiểm tra mật khẩu mới không trùng với mật khẩu cũ."</t>
+  </si>
+  <si>
+    <t>AI đề xuất sử dụng một biểu thức chính quy duy nhất ^(?=.*[a-z])(?=.*[A-Z])(?=.*\d)(?=.*[@$!%*?&amp;])[A-Za-z\d@$!%*?&amp;]{8,}$ và sử dụng hàm compare của thư viện bcrypt để so sánh trực tiếp mật khẩu mới với mã hash mật khẩu cũ trong controller của backend.</t>
+  </si>
+  <si>
+    <t>Quyết định cuối cùng và Lý do: Quyết định tách biệt logic xác thực: Giao diện (UI) xử lý checklist thời gian thực để định hướng tốt cho người dùng, Backend áp dụng Zod schema linh hoạt với tập ký tự đặc biệt mở rộng và so sánh bcrypt chống trùng lặp mật khẩu cũ.</t>
+  </si>
+  <si>
+    <t>Pattern Recognition</t>
+  </si>
+  <si>
+    <t>"Tại sao Mongoose lại trả về lỗi xác thực cho các tài liệu con (subdocuments) trống trong mảng 'addresses' khi cập nhật thông tin hồ sơ người dùng, mặc dù người dùng không hề chỉnh sửa địa chỉ của họ?"</t>
+  </si>
+  <si>
+    <t>AI trả lời rằng lỗi xảy ra vì trường addresses không được cấu hình required: false trong Mongoose schema, hoặc do request cập nhật đang gửi lên một đối tượng trống {}. AI khuyên nên sửa schema thành default: undefined cho mảng addresses.</t>
+  </si>
+  <si>
+    <t>Quyết định cuối cùng và Lý do: Quyết định áp dụng khai báo mảng tường minh kết hợp pre-validate hook làm sạch dữ liệu. Đây là giải pháp tối ưu giúp hệ thống tự phục hồi dữ liệu cũ mà không cần chạy migration database phức tạp hay làm mất cấu trúc mảng rỗng mặc định.</t>
   </si>
 </sst>
 </file>
@@ -103,7 +102,7 @@
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Aptos Narrow"/>
+      <name val="Arial"/>
       <family val="2"/>
       <charset val="163"/>
       <scheme val="minor"/>
@@ -112,7 +111,7 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Aptos Narrow"/>
+      <name val="Arial"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -507,102 +506,101 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EFBDDC7E-59F2-4CBB-B3D2-F6FB78F9E873}">
   <dimension ref="A1:F5"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="20.88671875" customWidth="1"/>
-    <col min="2" max="2" width="26.88671875" customWidth="1"/>
-    <col min="3" max="3" width="24.21875" customWidth="1"/>
-    <col min="4" max="4" width="25.5546875" customWidth="1"/>
+    <col min="1" max="1" width="20.875" customWidth="1"/>
+    <col min="2" max="2" width="26.875" customWidth="1"/>
+    <col min="3" max="3" width="24.25" customWidth="1"/>
+    <col min="4" max="4" width="25.5625" customWidth="1"/>
     <col min="5" max="5" width="45" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" ht="13.9" x14ac:dyDescent="0.35">
       <c r="A1" s="5" t="s">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>16</v>
+        <v>4</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="F1" s="1"/>
     </row>
-    <row r="2" spans="1:6" ht="72" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:6" ht="148.5" x14ac:dyDescent="0.35">
       <c r="A2" s="2">
         <v>1</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>1</v>
-      </c>
-      <c r="D2" s="6"/>
+        <v>5</v>
+      </c>
+      <c r="D2" s="6" t="s">
+        <v>6</v>
+      </c>
       <c r="E2" s="4" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:6" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:6" ht="135" x14ac:dyDescent="0.35">
       <c r="A3" s="2">
         <v>2</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="C3" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="D3" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="E3" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="D3" s="6"/>
-      <c r="E3" s="4" t="s">
-        <v>13</v>
-      </c>
     </row>
-    <row r="4" spans="1:6" ht="72" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:6" ht="121.5" x14ac:dyDescent="0.35">
       <c r="A4" s="2">
         <v>3</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>3</v>
+        <v>13</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>4</v>
-      </c>
-      <c r="D4" s="6"/>
+        <v>14</v>
+      </c>
+      <c r="D4" s="6" t="s">
+        <v>15</v>
+      </c>
       <c r="E4" s="4" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
     </row>
-    <row r="5" spans="1:6" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="A5" s="2">
-        <v>4</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="C5" s="6" t="s">
-        <v>6</v>
-      </c>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A5" s="2"/>
+      <c r="B5" s="3"/>
+      <c r="C5" s="6"/>
       <c r="D5" s="6"/>
-      <c r="E5" s="4" t="s">
-        <v>15</v>
-      </c>
+      <c r="E5" s="4"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{59E3EFE9-6FFB-49CC-BE69-0C0E36C6253E}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.35"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -611,7 +609,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{69A16565-6ACB-4DDB-B0C1-55C7722368A3}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.35"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -620,7 +618,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{323516A4-AE23-41CF-AD84-97A6064FC5FB}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.35"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -629,7 +627,7 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B38EFF89-9459-4552-9A9D-015DA017CF48}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.35"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>